<commit_message>
Stabilized Functional Fixes - up to spider spindle
</commit_message>
<xml_diff>
--- a/Doc/Master Data for Pilot Models.xlsx
+++ b/Doc/Master Data for Pilot Models.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\Workspace\Watchcase Tracker Titan\Doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\Workspace\Watchcase\TTT-Jan2026\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B744196-9473-44B1-BFFE-1342A980EFC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DB9538A-AD70-42AA-9F67-598B7EC78F69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pilot Models and Variants list " sheetId="1" r:id="rId1"/>
@@ -797,7 +797,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -849,8 +849,16 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -881,8 +889,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="65">
+  <borders count="71">
     <border>
       <left/>
       <right/>
@@ -1235,21 +1249,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -1603,166 +1602,245 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
         <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="-0.249977111117893"/>
+      </left>
+      <right style="thin">
+        <color theme="4" tint="-0.249977111117893"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="-0.249977111117893"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="-0.249977111117893"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="-0.249977111117893"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="-0.249977111117893"/>
       </right>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color theme="4" tint="-0.249977111117893"/>
       </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
+      <top/>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color theme="4" tint="-0.249977111117893"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color theme="4" tint="-0.249977111117893"/>
       </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
+      <right/>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color theme="4" tint="-0.249977111117893"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="-0.249977111117893"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="-0.249977111117893"/>
+      </left>
+      <right/>
+      <top/>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color theme="4" tint="-0.249977111117893"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color theme="4" tint="-0.249977111117893"/>
       </right>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color theme="4" tint="-0.249977111117893"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1818,91 +1896,82 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1911,36 +1980,33 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1956,67 +2022,64 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2029,47 +2092,77 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2357,20 +2450,28 @@
     <col min="1" max="1" width="15.81640625" style="12" customWidth="1"/>
     <col min="2" max="2" width="11.54296875" style="12" customWidth="1"/>
     <col min="3" max="3" width="10.453125" style="12" customWidth="1"/>
-    <col min="4" max="4" width="9.7265625" style="12" customWidth="1"/>
-    <col min="5" max="5" width="15.81640625" style="12" customWidth="1"/>
-    <col min="6" max="6" width="6.36328125" style="12" customWidth="1"/>
-    <col min="7" max="7" width="9.36328125" style="12" customWidth="1"/>
-    <col min="8" max="12" width="15.81640625" style="12" customWidth="1"/>
-    <col min="13" max="13" width="13.1796875" style="12" customWidth="1"/>
-    <col min="14" max="14" width="7.08984375" style="12" customWidth="1"/>
-    <col min="15" max="15" width="11.08984375" style="12" customWidth="1"/>
-    <col min="16" max="20" width="15.81640625" style="12" customWidth="1"/>
+    <col min="4" max="4" width="12.7265625" style="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.1796875" style="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.6328125" style="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12" style="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.54296875" style="12" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16" style="12" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.1796875" style="12" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.1796875" style="12" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.81640625" style="12" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.36328125" style="12" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.1796875" style="12" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.7265625" style="12" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.54296875" style="12" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.1796875" style="12" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="19.453125" style="12" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="19.90625" style="12" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="15.81640625" style="12" customWidth="1"/>
     <col min="21" max="16384" width="8.7265625" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="103" customFormat="1" ht="50.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="102" t="s">
+    <row r="1" spans="1:20" s="86" customFormat="1" ht="50.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="85" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -2435,22 +2536,22 @@
       <c r="A2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="87" t="s">
+      <c r="B2" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C2" s="87" t="s">
+      <c r="C2" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D2" s="87" t="s">
+      <c r="D2" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="88" t="s">
+      <c r="E2" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F2" s="89">
-        <v>30</v>
-      </c>
-      <c r="G2" s="88" t="s">
+      <c r="F2" s="84">
+        <v>30</v>
+      </c>
+      <c r="G2" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H2" s="4" t="s">
@@ -2497,22 +2598,22 @@
       <c r="A3" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="87" t="s">
+      <c r="B3" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C3" s="87" t="s">
+      <c r="C3" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D3" s="87" t="s">
+      <c r="D3" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="88" t="s">
+      <c r="E3" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F3" s="89">
-        <v>30</v>
-      </c>
-      <c r="G3" s="88" t="s">
+      <c r="F3" s="84">
+        <v>30</v>
+      </c>
+      <c r="G3" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H3" s="7" t="s">
@@ -2559,22 +2660,22 @@
       <c r="A4" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="87" t="s">
+      <c r="B4" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C4" s="87" t="s">
+      <c r="C4" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D4" s="87" t="s">
+      <c r="D4" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="88" t="s">
+      <c r="E4" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F4" s="89">
-        <v>30</v>
-      </c>
-      <c r="G4" s="88" t="s">
+      <c r="F4" s="84">
+        <v>30</v>
+      </c>
+      <c r="G4" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H4" s="7" t="s">
@@ -2621,22 +2722,22 @@
       <c r="A5" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="87" t="s">
+      <c r="B5" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C5" s="87" t="s">
+      <c r="C5" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D5" s="87" t="s">
+      <c r="D5" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="88" t="s">
+      <c r="E5" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F5" s="89">
-        <v>30</v>
-      </c>
-      <c r="G5" s="88" t="s">
+      <c r="F5" s="84">
+        <v>30</v>
+      </c>
+      <c r="G5" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H5" s="7" t="s">
@@ -2683,22 +2784,22 @@
       <c r="A6" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="87" t="s">
+      <c r="B6" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C6" s="87" t="s">
+      <c r="C6" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D6" s="87" t="s">
+      <c r="D6" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="88" t="s">
+      <c r="E6" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F6" s="89">
-        <v>30</v>
-      </c>
-      <c r="G6" s="88" t="s">
+      <c r="F6" s="84">
+        <v>30</v>
+      </c>
+      <c r="G6" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H6" s="7" t="s">
@@ -2745,22 +2846,22 @@
       <c r="A7" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="87" t="s">
+      <c r="B7" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C7" s="87" t="s">
+      <c r="C7" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D7" s="87" t="s">
+      <c r="D7" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="88" t="s">
+      <c r="E7" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F7" s="89">
-        <v>30</v>
-      </c>
-      <c r="G7" s="88" t="s">
+      <c r="F7" s="84">
+        <v>30</v>
+      </c>
+      <c r="G7" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H7" s="7" t="s">
@@ -2807,22 +2908,22 @@
       <c r="A8" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="87" t="s">
+      <c r="B8" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C8" s="87" t="s">
+      <c r="C8" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D8" s="87" t="s">
+      <c r="D8" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="88" t="s">
+      <c r="E8" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F8" s="89">
-        <v>30</v>
-      </c>
-      <c r="G8" s="88" t="s">
+      <c r="F8" s="84">
+        <v>30</v>
+      </c>
+      <c r="G8" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H8" s="7" t="s">
@@ -2869,22 +2970,22 @@
       <c r="A9" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B9" s="87" t="s">
+      <c r="B9" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C9" s="87" t="s">
+      <c r="C9" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D9" s="87" t="s">
+      <c r="D9" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="88" t="s">
+      <c r="E9" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F9" s="89">
-        <v>30</v>
-      </c>
-      <c r="G9" s="88" t="s">
+      <c r="F9" s="84">
+        <v>30</v>
+      </c>
+      <c r="G9" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H9" s="7" t="s">
@@ -2931,22 +3032,22 @@
       <c r="A10" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B10" s="87" t="s">
+      <c r="B10" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C10" s="87" t="s">
+      <c r="C10" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D10" s="87" t="s">
+      <c r="D10" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E10" s="88" t="s">
+      <c r="E10" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F10" s="89">
-        <v>30</v>
-      </c>
-      <c r="G10" s="88" t="s">
+      <c r="F10" s="84">
+        <v>30</v>
+      </c>
+      <c r="G10" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H10" s="7" t="s">
@@ -2993,22 +3094,22 @@
       <c r="A11" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="87" t="s">
+      <c r="B11" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C11" s="87" t="s">
+      <c r="C11" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D11" s="87" t="s">
+      <c r="D11" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E11" s="88" t="s">
+      <c r="E11" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F11" s="89">
-        <v>30</v>
-      </c>
-      <c r="G11" s="88" t="s">
+      <c r="F11" s="84">
+        <v>30</v>
+      </c>
+      <c r="G11" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H11" s="7" t="s">
@@ -3055,22 +3156,22 @@
       <c r="A12" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B12" s="87" t="s">
+      <c r="B12" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C12" s="87" t="s">
+      <c r="C12" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D12" s="87" t="s">
+      <c r="D12" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="88" t="s">
+      <c r="E12" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F12" s="89">
-        <v>30</v>
-      </c>
-      <c r="G12" s="88" t="s">
+      <c r="F12" s="84">
+        <v>30</v>
+      </c>
+      <c r="G12" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H12" s="7" t="s">
@@ -3117,22 +3218,22 @@
       <c r="A13" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B13" s="87" t="s">
+      <c r="B13" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C13" s="87" t="s">
+      <c r="C13" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D13" s="87" t="s">
+      <c r="D13" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E13" s="88" t="s">
+      <c r="E13" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F13" s="89">
-        <v>30</v>
-      </c>
-      <c r="G13" s="88" t="s">
+      <c r="F13" s="84">
+        <v>30</v>
+      </c>
+      <c r="G13" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H13" s="7" t="s">
@@ -3179,22 +3280,22 @@
       <c r="A14" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="87" t="s">
+      <c r="B14" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C14" s="87" t="s">
+      <c r="C14" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D14" s="87" t="s">
+      <c r="D14" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E14" s="88" t="s">
+      <c r="E14" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F14" s="89">
-        <v>30</v>
-      </c>
-      <c r="G14" s="88" t="s">
+      <c r="F14" s="84">
+        <v>30</v>
+      </c>
+      <c r="G14" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H14" s="7" t="s">
@@ -3241,22 +3342,22 @@
       <c r="A15" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="87" t="s">
+      <c r="B15" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C15" s="87" t="s">
+      <c r="C15" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D15" s="87" t="s">
+      <c r="D15" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="88" t="s">
+      <c r="E15" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F15" s="89">
-        <v>30</v>
-      </c>
-      <c r="G15" s="88" t="s">
+      <c r="F15" s="84">
+        <v>30</v>
+      </c>
+      <c r="G15" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H15" s="7" t="s">
@@ -3303,22 +3404,22 @@
       <c r="A16" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B16" s="87" t="s">
+      <c r="B16" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C16" s="87" t="s">
+      <c r="C16" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D16" s="87" t="s">
+      <c r="D16" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E16" s="88" t="s">
+      <c r="E16" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F16" s="89">
-        <v>30</v>
-      </c>
-      <c r="G16" s="88" t="s">
+      <c r="F16" s="84">
+        <v>30</v>
+      </c>
+      <c r="G16" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H16" s="7" t="s">
@@ -3365,22 +3466,22 @@
       <c r="A17" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B17" s="87" t="s">
+      <c r="B17" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C17" s="87" t="s">
+      <c r="C17" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D17" s="87" t="s">
+      <c r="D17" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E17" s="88" t="s">
+      <c r="E17" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F17" s="89">
-        <v>30</v>
-      </c>
-      <c r="G17" s="88" t="s">
+      <c r="F17" s="84">
+        <v>30</v>
+      </c>
+      <c r="G17" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H17" s="7" t="s">
@@ -3427,22 +3528,22 @@
       <c r="A18" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B18" s="87" t="s">
+      <c r="B18" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C18" s="87" t="s">
+      <c r="C18" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D18" s="87" t="s">
+      <c r="D18" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E18" s="88" t="s">
+      <c r="E18" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F18" s="89">
-        <v>30</v>
-      </c>
-      <c r="G18" s="88" t="s">
+      <c r="F18" s="84">
+        <v>30</v>
+      </c>
+      <c r="G18" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H18" s="7" t="s">
@@ -3489,22 +3590,22 @@
       <c r="A19" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="B19" s="87" t="s">
+      <c r="B19" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C19" s="87" t="s">
+      <c r="C19" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D19" s="87" t="s">
+      <c r="D19" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E19" s="88" t="s">
+      <c r="E19" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F19" s="89">
-        <v>30</v>
-      </c>
-      <c r="G19" s="88" t="s">
+      <c r="F19" s="84">
+        <v>30</v>
+      </c>
+      <c r="G19" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H19" s="7" t="s">
@@ -3551,22 +3652,22 @@
       <c r="A20" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B20" s="87" t="s">
+      <c r="B20" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C20" s="87" t="s">
+      <c r="C20" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D20" s="87" t="s">
+      <c r="D20" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E20" s="88" t="s">
+      <c r="E20" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F20" s="89">
-        <v>30</v>
-      </c>
-      <c r="G20" s="88" t="s">
+      <c r="F20" s="84">
+        <v>30</v>
+      </c>
+      <c r="G20" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H20" s="7" t="s">
@@ -3613,22 +3714,22 @@
       <c r="A21" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B21" s="87" t="s">
+      <c r="B21" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C21" s="87" t="s">
+      <c r="C21" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D21" s="87" t="s">
+      <c r="D21" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E21" s="88" t="s">
+      <c r="E21" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F21" s="89">
-        <v>30</v>
-      </c>
-      <c r="G21" s="88" t="s">
+      <c r="F21" s="84">
+        <v>30</v>
+      </c>
+      <c r="G21" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H21" s="7" t="s">
@@ -3675,22 +3776,22 @@
       <c r="A22" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="B22" s="87" t="s">
+      <c r="B22" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C22" s="87" t="s">
+      <c r="C22" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D22" s="87" t="s">
+      <c r="D22" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E22" s="88" t="s">
+      <c r="E22" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F22" s="89">
-        <v>30</v>
-      </c>
-      <c r="G22" s="88" t="s">
+      <c r="F22" s="84">
+        <v>30</v>
+      </c>
+      <c r="G22" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H22" s="7" t="s">
@@ -3737,22 +3838,22 @@
       <c r="A23" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B23" s="87" t="s">
+      <c r="B23" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C23" s="87" t="s">
+      <c r="C23" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D23" s="87" t="s">
+      <c r="D23" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E23" s="88" t="s">
+      <c r="E23" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F23" s="89">
-        <v>30</v>
-      </c>
-      <c r="G23" s="88" t="s">
+      <c r="F23" s="84">
+        <v>30</v>
+      </c>
+      <c r="G23" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H23" s="7" t="s">
@@ -3799,22 +3900,22 @@
       <c r="A24" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="B24" s="87" t="s">
+      <c r="B24" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C24" s="87" t="s">
+      <c r="C24" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D24" s="87" t="s">
+      <c r="D24" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E24" s="88" t="s">
+      <c r="E24" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F24" s="89">
-        <v>30</v>
-      </c>
-      <c r="G24" s="88" t="s">
+      <c r="F24" s="84">
+        <v>30</v>
+      </c>
+      <c r="G24" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H24" s="7" t="s">
@@ -3861,22 +3962,22 @@
       <c r="A25" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B25" s="87" t="s">
+      <c r="B25" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C25" s="87" t="s">
+      <c r="C25" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D25" s="87" t="s">
+      <c r="D25" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E25" s="88" t="s">
+      <c r="E25" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F25" s="89">
-        <v>30</v>
-      </c>
-      <c r="G25" s="88" t="s">
+      <c r="F25" s="84">
+        <v>30</v>
+      </c>
+      <c r="G25" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H25" s="7" t="s">
@@ -3923,22 +4024,22 @@
       <c r="A26" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B26" s="87" t="s">
+      <c r="B26" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C26" s="87" t="s">
+      <c r="C26" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D26" s="87" t="s">
+      <c r="D26" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E26" s="88" t="s">
+      <c r="E26" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F26" s="89">
-        <v>30</v>
-      </c>
-      <c r="G26" s="88" t="s">
+      <c r="F26" s="84">
+        <v>30</v>
+      </c>
+      <c r="G26" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H26" s="7" t="s">
@@ -3985,22 +4086,22 @@
       <c r="A27" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="B27" s="87" t="s">
+      <c r="B27" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C27" s="87" t="s">
+      <c r="C27" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D27" s="87" t="s">
+      <c r="D27" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E27" s="88" t="s">
+      <c r="E27" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F27" s="89">
-        <v>30</v>
-      </c>
-      <c r="G27" s="88" t="s">
+      <c r="F27" s="84">
+        <v>30</v>
+      </c>
+      <c r="G27" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H27" s="7" t="s">
@@ -4047,22 +4148,22 @@
       <c r="A28" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B28" s="87" t="s">
+      <c r="B28" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C28" s="87" t="s">
+      <c r="C28" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D28" s="87" t="s">
+      <c r="D28" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E28" s="88" t="s">
+      <c r="E28" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F28" s="89">
-        <v>30</v>
-      </c>
-      <c r="G28" s="88" t="s">
+      <c r="F28" s="84">
+        <v>30</v>
+      </c>
+      <c r="G28" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H28" s="7" t="s">
@@ -4109,22 +4210,22 @@
       <c r="A29" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="B29" s="87" t="s">
+      <c r="B29" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C29" s="87" t="s">
+      <c r="C29" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D29" s="87" t="s">
+      <c r="D29" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E29" s="88" t="s">
+      <c r="E29" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F29" s="89">
-        <v>30</v>
-      </c>
-      <c r="G29" s="88" t="s">
+      <c r="F29" s="84">
+        <v>30</v>
+      </c>
+      <c r="G29" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H29" s="7" t="s">
@@ -4171,22 +4272,22 @@
       <c r="A30" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B30" s="87" t="s">
+      <c r="B30" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C30" s="87" t="s">
+      <c r="C30" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D30" s="87" t="s">
+      <c r="D30" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E30" s="88" t="s">
+      <c r="E30" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F30" s="89">
-        <v>30</v>
-      </c>
-      <c r="G30" s="88" t="s">
+      <c r="F30" s="84">
+        <v>30</v>
+      </c>
+      <c r="G30" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H30" s="7" t="s">
@@ -4233,22 +4334,22 @@
       <c r="A31" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="B31" s="87" t="s">
+      <c r="B31" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C31" s="87" t="s">
+      <c r="C31" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D31" s="87" t="s">
+      <c r="D31" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E31" s="88" t="s">
+      <c r="E31" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F31" s="89">
-        <v>30</v>
-      </c>
-      <c r="G31" s="88" t="s">
+      <c r="F31" s="84">
+        <v>30</v>
+      </c>
+      <c r="G31" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H31" s="7" t="s">
@@ -4295,22 +4396,22 @@
       <c r="A32" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="B32" s="87" t="s">
+      <c r="B32" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C32" s="87" t="s">
+      <c r="C32" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D32" s="87" t="s">
+      <c r="D32" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E32" s="88" t="s">
+      <c r="E32" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F32" s="89">
-        <v>30</v>
-      </c>
-      <c r="G32" s="88" t="s">
+      <c r="F32" s="84">
+        <v>30</v>
+      </c>
+      <c r="G32" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H32" s="7" t="s">
@@ -4357,22 +4458,22 @@
       <c r="A33" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="B33" s="87" t="s">
+      <c r="B33" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C33" s="87" t="s">
+      <c r="C33" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D33" s="87" t="s">
+      <c r="D33" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E33" s="88" t="s">
+      <c r="E33" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F33" s="89">
-        <v>30</v>
-      </c>
-      <c r="G33" s="88" t="s">
+      <c r="F33" s="84">
+        <v>30</v>
+      </c>
+      <c r="G33" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H33" s="7" t="s">
@@ -4419,22 +4520,22 @@
       <c r="A34" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="B34" s="87" t="s">
+      <c r="B34" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D34" s="87" t="s">
+      <c r="D34" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E34" s="88" t="s">
+      <c r="E34" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F34" s="89">
-        <v>30</v>
-      </c>
-      <c r="G34" s="88" t="s">
+      <c r="F34" s="84">
+        <v>30</v>
+      </c>
+      <c r="G34" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H34" s="7" t="s">
@@ -4481,22 +4582,22 @@
       <c r="A35" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="B35" s="87" t="s">
+      <c r="B35" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C35" s="87" t="s">
+      <c r="C35" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D35" s="87" t="s">
+      <c r="D35" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E35" s="88" t="s">
+      <c r="E35" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F35" s="89">
-        <v>30</v>
-      </c>
-      <c r="G35" s="88" t="s">
+      <c r="F35" s="84">
+        <v>30</v>
+      </c>
+      <c r="G35" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H35" s="7" t="s">
@@ -4543,22 +4644,22 @@
       <c r="A36" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B36" s="87" t="s">
+      <c r="B36" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C36" s="87" t="s">
+      <c r="C36" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D36" s="87" t="s">
+      <c r="D36" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E36" s="88" t="s">
+      <c r="E36" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F36" s="89">
-        <v>30</v>
-      </c>
-      <c r="G36" s="88" t="s">
+      <c r="F36" s="84">
+        <v>30</v>
+      </c>
+      <c r="G36" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H36" s="7" t="s">
@@ -4605,22 +4706,22 @@
       <c r="A37" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="B37" s="87" t="s">
+      <c r="B37" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C37" s="87" t="s">
+      <c r="C37" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D37" s="87" t="s">
+      <c r="D37" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E37" s="88" t="s">
+      <c r="E37" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F37" s="89">
-        <v>30</v>
-      </c>
-      <c r="G37" s="88" t="s">
+      <c r="F37" s="84">
+        <v>30</v>
+      </c>
+      <c r="G37" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H37" s="7" t="s">
@@ -4667,22 +4768,22 @@
       <c r="A38" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B38" s="87" t="s">
+      <c r="B38" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C38" s="87" t="s">
+      <c r="C38" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D38" s="87" t="s">
+      <c r="D38" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E38" s="88" t="s">
+      <c r="E38" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F38" s="89">
-        <v>30</v>
-      </c>
-      <c r="G38" s="88" t="s">
+      <c r="F38" s="84">
+        <v>30</v>
+      </c>
+      <c r="G38" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H38" s="7" t="s">
@@ -4729,22 +4830,22 @@
       <c r="A39" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B39" s="87" t="s">
+      <c r="B39" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C39" s="87" t="s">
+      <c r="C39" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D39" s="87" t="s">
+      <c r="D39" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E39" s="88" t="s">
+      <c r="E39" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F39" s="89">
-        <v>30</v>
-      </c>
-      <c r="G39" s="88" t="s">
+      <c r="F39" s="84">
+        <v>30</v>
+      </c>
+      <c r="G39" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H39" s="7" t="s">
@@ -4791,22 +4892,22 @@
       <c r="A40" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="B40" s="87" t="s">
+      <c r="B40" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C40" s="87" t="s">
+      <c r="C40" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D40" s="87" t="s">
+      <c r="D40" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E40" s="88" t="s">
+      <c r="E40" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F40" s="89">
-        <v>30</v>
-      </c>
-      <c r="G40" s="88" t="s">
+      <c r="F40" s="84">
+        <v>30</v>
+      </c>
+      <c r="G40" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H40" s="7" t="s">
@@ -4853,22 +4954,22 @@
       <c r="A41" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B41" s="87" t="s">
+      <c r="B41" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C41" s="87" t="s">
+      <c r="C41" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D41" s="87" t="s">
+      <c r="D41" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E41" s="88" t="s">
+      <c r="E41" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F41" s="89">
-        <v>30</v>
-      </c>
-      <c r="G41" s="88" t="s">
+      <c r="F41" s="84">
+        <v>30</v>
+      </c>
+      <c r="G41" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H41" s="7" t="s">
@@ -4915,22 +5016,22 @@
       <c r="A42" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="B42" s="87" t="s">
+      <c r="B42" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C42" s="87" t="s">
+      <c r="C42" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D42" s="87" t="s">
+      <c r="D42" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E42" s="88" t="s">
+      <c r="E42" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F42" s="89">
-        <v>30</v>
-      </c>
-      <c r="G42" s="88" t="s">
+      <c r="F42" s="84">
+        <v>30</v>
+      </c>
+      <c r="G42" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H42" s="7" t="s">
@@ -4977,22 +5078,22 @@
       <c r="A43" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="B43" s="87" t="s">
+      <c r="B43" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C43" s="87" t="s">
+      <c r="C43" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D43" s="87" t="s">
+      <c r="D43" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E43" s="88" t="s">
+      <c r="E43" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F43" s="89">
-        <v>30</v>
-      </c>
-      <c r="G43" s="88" t="s">
+      <c r="F43" s="84">
+        <v>30</v>
+      </c>
+      <c r="G43" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H43" s="7" t="s">
@@ -5039,22 +5140,22 @@
       <c r="A44" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="B44" s="87" t="s">
+      <c r="B44" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C44" s="87" t="s">
+      <c r="C44" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D44" s="87" t="s">
+      <c r="D44" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E44" s="88" t="s">
+      <c r="E44" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F44" s="89">
-        <v>30</v>
-      </c>
-      <c r="G44" s="88" t="s">
+      <c r="F44" s="84">
+        <v>30</v>
+      </c>
+      <c r="G44" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H44" s="7" t="s">
@@ -5101,22 +5202,22 @@
       <c r="A45" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="B45" s="87" t="s">
+      <c r="B45" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C45" s="87" t="s">
+      <c r="C45" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D45" s="87" t="s">
+      <c r="D45" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E45" s="88" t="s">
+      <c r="E45" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F45" s="89">
-        <v>30</v>
-      </c>
-      <c r="G45" s="88" t="s">
+      <c r="F45" s="84">
+        <v>30</v>
+      </c>
+      <c r="G45" s="83" t="s">
         <v>253</v>
       </c>
       <c r="H45" s="10" t="s">
@@ -5160,322 +5261,322 @@
       </c>
     </row>
     <row r="46" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="B46" s="87" t="s">
+      <c r="B46" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C46" s="87" t="s">
+      <c r="C46" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D46" s="87" t="s">
+      <c r="D46" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E46" s="88" t="s">
+      <c r="E46" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F46" s="89">
-        <v>30</v>
-      </c>
-      <c r="G46" s="88" t="s">
+      <c r="F46" s="84">
+        <v>30</v>
+      </c>
+      <c r="G46" s="83" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="47" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="B47" s="87" t="s">
+      <c r="B47" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C47" s="87" t="s">
+      <c r="C47" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D47" s="87" t="s">
+      <c r="D47" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E47" s="88" t="s">
+      <c r="E47" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F47" s="89">
-        <v>30</v>
-      </c>
-      <c r="G47" s="88" t="s">
+      <c r="F47" s="84">
+        <v>30</v>
+      </c>
+      <c r="G47" s="83" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="48" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="B48" s="87" t="s">
+      <c r="B48" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C48" s="87" t="s">
+      <c r="C48" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D48" s="87" t="s">
+      <c r="D48" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E48" s="88" t="s">
+      <c r="E48" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F48" s="89">
-        <v>30</v>
-      </c>
-      <c r="G48" s="88" t="s">
+      <c r="F48" s="84">
+        <v>30</v>
+      </c>
+      <c r="G48" s="83" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="49" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B49" s="87" t="s">
+      <c r="B49" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C49" s="87" t="s">
+      <c r="C49" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D49" s="87" t="s">
+      <c r="D49" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E49" s="88" t="s">
+      <c r="E49" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F49" s="89">
-        <v>30</v>
-      </c>
-      <c r="G49" s="88" t="s">
+      <c r="F49" s="84">
+        <v>30</v>
+      </c>
+      <c r="G49" s="83" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="50" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B50" s="87" t="s">
+      <c r="B50" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C50" s="87" t="s">
+      <c r="C50" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D50" s="87" t="s">
+      <c r="D50" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E50" s="88" t="s">
+      <c r="E50" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F50" s="89">
-        <v>30</v>
-      </c>
-      <c r="G50" s="88" t="s">
+      <c r="F50" s="84">
+        <v>30</v>
+      </c>
+      <c r="G50" s="83" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="51" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B51" s="87" t="s">
+      <c r="B51" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C51" s="87" t="s">
+      <c r="C51" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D51" s="87" t="s">
+      <c r="D51" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E51" s="88" t="s">
+      <c r="E51" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F51" s="89">
-        <v>30</v>
-      </c>
-      <c r="G51" s="88" t="s">
+      <c r="F51" s="84">
+        <v>30</v>
+      </c>
+      <c r="G51" s="83" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="52" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B52" s="87" t="s">
+      <c r="B52" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C52" s="87" t="s">
+      <c r="C52" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D52" s="87" t="s">
+      <c r="D52" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E52" s="88" t="s">
+      <c r="E52" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F52" s="89">
-        <v>30</v>
-      </c>
-      <c r="G52" s="88" t="s">
+      <c r="F52" s="84">
+        <v>30</v>
+      </c>
+      <c r="G52" s="83" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="53" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B53" s="87" t="s">
+      <c r="B53" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C53" s="87" t="s">
+      <c r="C53" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D53" s="87" t="s">
+      <c r="D53" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E53" s="88" t="s">
+      <c r="E53" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F53" s="89">
-        <v>30</v>
-      </c>
-      <c r="G53" s="88" t="s">
+      <c r="F53" s="84">
+        <v>30</v>
+      </c>
+      <c r="G53" s="83" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="54" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B54" s="87" t="s">
+      <c r="B54" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C54" s="87" t="s">
+      <c r="C54" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D54" s="87" t="s">
+      <c r="D54" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E54" s="88" t="s">
+      <c r="E54" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F54" s="89">
-        <v>30</v>
-      </c>
-      <c r="G54" s="88" t="s">
+      <c r="F54" s="84">
+        <v>30</v>
+      </c>
+      <c r="G54" s="83" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="55" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B55" s="87" t="s">
+      <c r="B55" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C55" s="87" t="s">
+      <c r="C55" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D55" s="87" t="s">
+      <c r="D55" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E55" s="88" t="s">
+      <c r="E55" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F55" s="89">
-        <v>30</v>
-      </c>
-      <c r="G55" s="88" t="s">
+      <c r="F55" s="84">
+        <v>30</v>
+      </c>
+      <c r="G55" s="83" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="56" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B56" s="87" t="s">
+      <c r="B56" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C56" s="87" t="s">
+      <c r="C56" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D56" s="87" t="s">
+      <c r="D56" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E56" s="88" t="s">
+      <c r="E56" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F56" s="89">
-        <v>30</v>
-      </c>
-      <c r="G56" s="88" t="s">
+      <c r="F56" s="84">
+        <v>30</v>
+      </c>
+      <c r="G56" s="83" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="57" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B57" s="87" t="s">
+      <c r="B57" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C57" s="87" t="s">
+      <c r="C57" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D57" s="87" t="s">
+      <c r="D57" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E57" s="88" t="s">
+      <c r="E57" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F57" s="89">
-        <v>30</v>
-      </c>
-      <c r="G57" s="88" t="s">
+      <c r="F57" s="84">
+        <v>30</v>
+      </c>
+      <c r="G57" s="83" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="58" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B58" s="87" t="s">
+      <c r="B58" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C58" s="87" t="s">
+      <c r="C58" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D58" s="87" t="s">
+      <c r="D58" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E58" s="88" t="s">
+      <c r="E58" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F58" s="89">
-        <v>30</v>
-      </c>
-      <c r="G58" s="88" t="s">
+      <c r="F58" s="84">
+        <v>30</v>
+      </c>
+      <c r="G58" s="83" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B59" s="87" t="s">
+      <c r="B59" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C59" s="87" t="s">
+      <c r="C59" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D59" s="87" t="s">
+      <c r="D59" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E59" s="88" t="s">
+      <c r="E59" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F59" s="89">
-        <v>30</v>
-      </c>
-      <c r="G59" s="88" t="s">
+      <c r="F59" s="84">
+        <v>30</v>
+      </c>
+      <c r="G59" s="83" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="60" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B60" s="87" t="s">
+      <c r="B60" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C60" s="87" t="s">
+      <c r="C60" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D60" s="87" t="s">
+      <c r="D60" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E60" s="88" t="s">
+      <c r="E60" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F60" s="89">
-        <v>30</v>
-      </c>
-      <c r="G60" s="88" t="s">
+      <c r="F60" s="84">
+        <v>30</v>
+      </c>
+      <c r="G60" s="83" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="61" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B61" s="87" t="s">
+      <c r="B61" s="82" t="s">
         <v>251</v>
       </c>
-      <c r="C61" s="87" t="s">
+      <c r="C61" s="82" t="s">
         <v>252</v>
       </c>
-      <c r="D61" s="87" t="s">
+      <c r="D61" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="E61" s="88" t="s">
+      <c r="E61" s="83" t="s">
         <v>249</v>
       </c>
-      <c r="F61" s="89">
-        <v>30</v>
-      </c>
-      <c r="G61" s="88" t="s">
+      <c r="F61" s="84">
+        <v>30</v>
+      </c>
+      <c r="G61" s="83" t="s">
         <v>253</v>
       </c>
     </row>
@@ -5501,7 +5602,11 @@
     <col min="11" max="12" width="17.54296875" style="12" customWidth="1"/>
     <col min="13" max="13" width="12.54296875" style="12" customWidth="1"/>
     <col min="14" max="14" width="22.26953125" style="12" customWidth="1"/>
-    <col min="15" max="27" width="17.54296875" style="12" customWidth="1"/>
+    <col min="15" max="23" width="17.54296875" style="12" customWidth="1"/>
+    <col min="24" max="24" width="10.54296875" style="12" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="15.26953125" style="12" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="8.7265625" style="12" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="17.54296875" style="12" customWidth="1"/>
     <col min="28" max="28" width="6.90625" style="12" customWidth="1"/>
     <col min="29" max="30" width="17.54296875" style="12" customWidth="1"/>
     <col min="31" max="31" width="7.26953125" style="12" customWidth="1"/>
@@ -5516,169 +5621,169 @@
   <sheetData>
     <row r="1" spans="5:42" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="5:42" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="E2" s="86" t="s">
+      <c r="E2" s="81" t="s">
         <v>247</v>
       </c>
-      <c r="G2" s="96" t="s">
+      <c r="G2" s="93" t="s">
         <v>103</v>
       </c>
-      <c r="H2" s="97"/>
+      <c r="H2" s="94"/>
       <c r="I2" s="14"/>
-      <c r="J2" s="90" t="s">
+      <c r="J2" s="87" t="s">
         <v>104</v>
       </c>
-      <c r="K2" s="92"/>
+      <c r="K2" s="89"/>
       <c r="L2" s="14"/>
-      <c r="M2" s="90" t="s">
+      <c r="M2" s="87" t="s">
         <v>105</v>
       </c>
-      <c r="N2" s="92"/>
+      <c r="N2" s="89"/>
       <c r="O2" s="13"/>
-      <c r="P2" s="98" t="s">
+      <c r="P2" s="95" t="s">
         <v>106</v>
       </c>
-      <c r="Q2" s="100" t="s">
+      <c r="Q2" s="97" t="s">
         <v>107</v>
       </c>
-      <c r="R2" s="91" t="s">
+      <c r="R2" s="88" t="s">
         <v>108</v>
       </c>
-      <c r="S2" s="91"/>
-      <c r="T2" s="91"/>
-      <c r="U2" s="92"/>
+      <c r="S2" s="88"/>
+      <c r="T2" s="88"/>
+      <c r="U2" s="89"/>
       <c r="V2" s="14"/>
       <c r="W2" s="14"/>
-      <c r="X2" s="90" t="s">
+      <c r="X2" s="99" t="s">
         <v>109</v>
       </c>
-      <c r="Y2" s="91"/>
-      <c r="Z2" s="92"/>
+      <c r="Y2" s="99"/>
+      <c r="Z2" s="99"/>
       <c r="AA2" s="14"/>
-      <c r="AB2" s="70" t="s">
+      <c r="AB2" s="65" t="s">
         <v>116</v>
       </c>
-      <c r="AC2" s="71" t="s">
+      <c r="AC2" s="66" t="s">
         <v>11</v>
       </c>
       <c r="AD2" s="14"/>
-      <c r="AE2" s="72" t="s">
+      <c r="AE2" s="67" t="s">
         <v>116</v>
       </c>
-      <c r="AF2" s="73" t="s">
+      <c r="AF2" s="68" t="s">
         <v>8</v>
       </c>
-      <c r="AG2" s="74" t="s">
+      <c r="AG2" s="69" t="s">
         <v>117</v>
       </c>
       <c r="AH2" s="14"/>
-      <c r="AI2" s="75" t="s">
+      <c r="AI2" s="70" t="s">
         <v>118</v>
       </c>
       <c r="AJ2" s="14"/>
-      <c r="AK2" s="82" t="s">
+      <c r="AK2" s="77" t="s">
         <v>116</v>
       </c>
-      <c r="AL2" s="74" t="s">
+      <c r="AL2" s="69" t="s">
         <v>119</v>
       </c>
       <c r="AM2" s="14"/>
-      <c r="AN2" s="82" t="s">
+      <c r="AN2" s="77" t="s">
         <v>116</v>
       </c>
-      <c r="AO2" s="74" t="s">
+      <c r="AO2" s="69" t="s">
         <v>120</v>
       </c>
       <c r="AP2" s="14"/>
     </row>
     <row r="3" spans="5:42" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="E3" s="23" t="s">
+      <c r="E3" s="21" t="s">
         <v>248</v>
       </c>
-      <c r="G3" s="63" t="s">
+      <c r="G3" s="59" t="s">
         <v>110</v>
       </c>
-      <c r="H3" s="64" t="s">
+      <c r="H3" s="60" t="s">
         <v>111</v>
       </c>
       <c r="I3" s="14"/>
-      <c r="J3" s="65" t="s">
+      <c r="J3" s="61" t="s">
         <v>110</v>
       </c>
-      <c r="K3" s="66" t="s">
+      <c r="K3" s="62" t="s">
         <v>111</v>
       </c>
       <c r="L3" s="14"/>
-      <c r="M3" s="68" t="s">
+      <c r="M3" s="64" t="s">
         <v>110</v>
       </c>
-      <c r="N3" s="67" t="s">
+      <c r="N3" s="63" t="s">
         <v>112</v>
       </c>
       <c r="O3" s="13"/>
-      <c r="P3" s="99"/>
-      <c r="Q3" s="101"/>
-      <c r="R3" s="60">
+      <c r="P3" s="96"/>
+      <c r="Q3" s="98"/>
+      <c r="R3" s="56">
         <v>0.65</v>
       </c>
-      <c r="S3" s="61">
+      <c r="S3" s="57">
         <v>1</v>
       </c>
-      <c r="T3" s="61">
+      <c r="T3" s="57">
         <v>1.5</v>
       </c>
-      <c r="U3" s="62">
+      <c r="U3" s="58">
         <v>2.5</v>
       </c>
       <c r="V3" s="14"/>
       <c r="W3" s="14"/>
-      <c r="X3" s="69" t="s">
+      <c r="X3" s="100" t="s">
         <v>113</v>
       </c>
-      <c r="Y3" s="61" t="s">
+      <c r="Y3" s="102" t="s">
         <v>114</v>
       </c>
-      <c r="Z3" s="62" t="s">
+      <c r="Z3" s="100" t="s">
         <v>115</v>
       </c>
       <c r="AA3" s="14"/>
-      <c r="AB3" s="22">
+      <c r="AB3" s="20">
         <v>1</v>
       </c>
-      <c r="AC3" s="24">
+      <c r="AC3" s="22">
         <v>70</v>
       </c>
       <c r="AD3" s="14"/>
-      <c r="AE3" s="57">
+      <c r="AE3" s="53">
         <v>1</v>
       </c>
-      <c r="AF3" s="58" t="s">
+      <c r="AF3" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="AG3" s="59" t="s">
+      <c r="AG3" s="55" t="s">
         <v>130</v>
       </c>
       <c r="AH3" s="14"/>
-      <c r="AI3" s="26" t="s">
+      <c r="AI3" s="24" t="s">
         <v>131</v>
       </c>
       <c r="AJ3" s="14"/>
-      <c r="AK3" s="80">
+      <c r="AK3" s="75">
         <v>1</v>
       </c>
-      <c r="AL3" s="81" t="s">
+      <c r="AL3" s="76" t="s">
         <v>132</v>
       </c>
       <c r="AM3" s="14"/>
-      <c r="AN3" s="80">
+      <c r="AN3" s="75">
         <v>1</v>
       </c>
-      <c r="AO3" s="83" t="s">
+      <c r="AO3" s="78" t="s">
         <v>133</v>
       </c>
       <c r="AP3" s="14"/>
     </row>
     <row r="4" spans="5:42" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E4" s="34" t="s">
+      <c r="E4" s="31" t="s">
         <v>249</v>
       </c>
       <c r="G4" s="16">
@@ -5705,322 +5810,322 @@
       <c r="P4" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="Q4" s="51">
+      <c r="Q4" s="47">
         <v>13</v>
       </c>
-      <c r="R4" s="20">
+      <c r="R4" s="19">
         <v>0</v>
       </c>
-      <c r="S4" s="20">
+      <c r="S4" s="19">
         <v>0</v>
       </c>
-      <c r="T4" s="20">
+      <c r="T4" s="19">
         <v>0</v>
       </c>
-      <c r="U4" s="48">
+      <c r="U4" s="44">
         <v>1</v>
       </c>
-      <c r="V4" s="93" t="s">
+      <c r="V4" s="90" t="s">
         <v>125</v>
       </c>
       <c r="W4" s="14"/>
-      <c r="X4" s="18" t="s">
+      <c r="X4" s="101" t="s">
         <v>126</v>
       </c>
-      <c r="Y4" s="19" t="s">
+      <c r="Y4" s="103" t="s">
         <v>127</v>
       </c>
-      <c r="Z4" s="21" t="s">
+      <c r="Z4" s="106" t="s">
         <v>128</v>
       </c>
       <c r="AA4" s="14"/>
-      <c r="AB4" s="33">
+      <c r="AB4" s="30">
         <v>2</v>
       </c>
-      <c r="AC4" s="35">
+      <c r="AC4" s="32">
         <v>98</v>
       </c>
       <c r="AD4" s="14"/>
-      <c r="AE4" s="52">
+      <c r="AE4" s="48">
         <v>2</v>
       </c>
-      <c r="AF4" s="25" t="s">
+      <c r="AF4" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="AG4" s="53" t="s">
+      <c r="AG4" s="49" t="s">
         <v>140</v>
       </c>
       <c r="AH4" s="14"/>
-      <c r="AI4" s="36" t="s">
+      <c r="AI4" s="33" t="s">
         <v>103</v>
       </c>
       <c r="AJ4" s="14"/>
-      <c r="AK4" s="76">
+      <c r="AK4" s="71">
         <v>2</v>
       </c>
-      <c r="AL4" s="77" t="s">
+      <c r="AL4" s="72" t="s">
         <v>141</v>
       </c>
       <c r="AM4" s="14"/>
-      <c r="AN4" s="76">
+      <c r="AN4" s="71">
         <v>2</v>
       </c>
-      <c r="AO4" s="84" t="s">
+      <c r="AO4" s="79" t="s">
         <v>142</v>
       </c>
       <c r="AP4" s="14"/>
     </row>
     <row r="5" spans="5:42" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="E5" s="42" t="s">
+      <c r="E5" s="38" t="s">
         <v>250</v>
       </c>
-      <c r="G5" s="28">
+      <c r="G5" s="26">
         <v>2</v>
       </c>
-      <c r="H5" s="29" t="s">
+      <c r="H5" s="27" t="s">
         <v>134</v>
       </c>
       <c r="I5" s="14"/>
-      <c r="J5" s="28">
+      <c r="J5" s="26">
         <v>2</v>
       </c>
-      <c r="K5" s="29" t="s">
+      <c r="K5" s="27" t="s">
         <v>135</v>
       </c>
       <c r="L5" s="14"/>
-      <c r="M5" s="28">
+      <c r="M5" s="26">
         <v>2</v>
       </c>
-      <c r="N5" s="29" t="s">
+      <c r="N5" s="27" t="s">
         <v>136</v>
       </c>
       <c r="O5" s="14"/>
-      <c r="P5" s="30" t="s">
+      <c r="P5" s="28" t="s">
         <v>137</v>
       </c>
-      <c r="Q5" s="27">
+      <c r="Q5" s="25">
         <v>20</v>
       </c>
-      <c r="R5" s="31">
+      <c r="R5" s="29">
         <v>0</v>
       </c>
-      <c r="S5" s="31">
+      <c r="S5" s="29">
         <v>0</v>
       </c>
-      <c r="T5" s="31">
+      <c r="T5" s="29">
         <v>1</v>
       </c>
-      <c r="U5" s="49">
+      <c r="U5" s="45">
         <v>1</v>
       </c>
-      <c r="V5" s="94"/>
+      <c r="V5" s="91"/>
       <c r="W5" s="14"/>
-      <c r="X5" s="30" t="s">
+      <c r="X5" s="101" t="s">
         <v>138</v>
       </c>
-      <c r="Y5" s="27"/>
-      <c r="Z5" s="32"/>
+      <c r="Y5" s="104"/>
+      <c r="Z5" s="107"/>
       <c r="AA5" s="14"/>
-      <c r="AB5" s="33">
+      <c r="AB5" s="30">
         <v>3</v>
       </c>
-      <c r="AC5" s="35">
+      <c r="AC5" s="32">
         <v>144</v>
       </c>
       <c r="AD5" s="14"/>
-      <c r="AE5" s="52">
+      <c r="AE5" s="48">
         <v>3</v>
       </c>
-      <c r="AF5" s="25" t="s">
+      <c r="AF5" s="23" t="s">
         <v>148</v>
       </c>
-      <c r="AG5" s="53" t="s">
+      <c r="AG5" s="49" t="s">
         <v>149</v>
       </c>
       <c r="AH5" s="14"/>
-      <c r="AI5" s="36" t="s">
+      <c r="AI5" s="33" t="s">
         <v>150</v>
       </c>
       <c r="AJ5" s="14"/>
-      <c r="AK5" s="76">
+      <c r="AK5" s="71">
         <v>3</v>
       </c>
-      <c r="AL5" s="77" t="s">
+      <c r="AL5" s="72" t="s">
         <v>151</v>
       </c>
       <c r="AM5" s="14"/>
-      <c r="AN5" s="76">
+      <c r="AN5" s="71">
         <v>3</v>
       </c>
-      <c r="AO5" s="84" t="s">
+      <c r="AO5" s="79" t="s">
         <v>152</v>
       </c>
       <c r="AP5" s="14"/>
     </row>
-    <row r="6" spans="5:42" ht="29" x14ac:dyDescent="0.35">
-      <c r="G6" s="28">
+    <row r="6" spans="5:42" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G6" s="26">
         <v>3</v>
       </c>
-      <c r="H6" s="29" t="s">
+      <c r="H6" s="27" t="s">
         <v>143</v>
       </c>
       <c r="I6" s="14"/>
-      <c r="J6" s="28">
+      <c r="J6" s="26">
         <v>3</v>
       </c>
-      <c r="K6" s="29" t="s">
+      <c r="K6" s="27" t="s">
         <v>144</v>
       </c>
       <c r="L6" s="14"/>
-      <c r="M6" s="28">
+      <c r="M6" s="26">
         <v>3</v>
       </c>
-      <c r="N6" s="29" t="s">
+      <c r="N6" s="27" t="s">
         <v>145</v>
       </c>
       <c r="O6" s="14"/>
-      <c r="P6" s="30" t="s">
+      <c r="P6" s="28" t="s">
         <v>146</v>
       </c>
-      <c r="Q6" s="27">
+      <c r="Q6" s="25">
         <v>32</v>
       </c>
-      <c r="R6" s="31">
+      <c r="R6" s="29">
         <v>0</v>
       </c>
-      <c r="S6" s="31">
+      <c r="S6" s="29">
         <v>1</v>
       </c>
-      <c r="T6" s="31">
+      <c r="T6" s="29">
         <v>1</v>
       </c>
-      <c r="U6" s="49">
+      <c r="U6" s="45">
         <v>2</v>
       </c>
-      <c r="V6" s="94"/>
+      <c r="V6" s="91"/>
       <c r="W6" s="14"/>
-      <c r="X6" s="30" t="s">
+      <c r="X6" s="101" t="s">
         <v>147</v>
       </c>
-      <c r="Y6" s="27"/>
-      <c r="Z6" s="32"/>
+      <c r="Y6" s="104"/>
+      <c r="Z6" s="107"/>
       <c r="AA6" s="14"/>
-      <c r="AB6" s="33">
+      <c r="AB6" s="30">
         <v>4</v>
       </c>
-      <c r="AC6" s="35">
+      <c r="AC6" s="32">
         <v>150</v>
       </c>
       <c r="AD6" s="14"/>
-      <c r="AE6" s="52">
+      <c r="AE6" s="48">
         <v>4</v>
       </c>
-      <c r="AF6" s="25" t="s">
+      <c r="AF6" s="23" t="s">
         <v>66</v>
       </c>
-      <c r="AG6" s="53" t="s">
+      <c r="AG6" s="49" t="s">
         <v>158</v>
       </c>
       <c r="AH6" s="14"/>
-      <c r="AI6" s="36" t="s">
+      <c r="AI6" s="33" t="s">
         <v>159</v>
       </c>
       <c r="AJ6" s="14"/>
-      <c r="AK6" s="76">
+      <c r="AK6" s="71">
         <v>4</v>
       </c>
-      <c r="AL6" s="77" t="s">
+      <c r="AL6" s="72" t="s">
         <v>160</v>
       </c>
       <c r="AM6" s="14"/>
-      <c r="AN6" s="76">
+      <c r="AN6" s="71">
         <v>4</v>
       </c>
-      <c r="AO6" s="84" t="s">
+      <c r="AO6" s="79" t="s">
         <v>161</v>
       </c>
       <c r="AP6" s="14"/>
     </row>
     <row r="7" spans="5:42" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="G7" s="37">
+      <c r="G7" s="34">
         <v>4</v>
       </c>
-      <c r="H7" s="47" t="s">
+      <c r="H7" s="43" t="s">
         <v>153</v>
       </c>
       <c r="I7" s="14"/>
-      <c r="J7" s="28">
+      <c r="J7" s="26">
         <v>4</v>
       </c>
-      <c r="K7" s="29" t="s">
+      <c r="K7" s="27" t="s">
         <v>154</v>
       </c>
       <c r="L7" s="14"/>
-      <c r="M7" s="28">
+      <c r="M7" s="26">
         <v>4</v>
       </c>
-      <c r="N7" s="29" t="s">
+      <c r="N7" s="27" t="s">
         <v>155</v>
       </c>
       <c r="O7" s="14"/>
-      <c r="P7" s="30" t="s">
+      <c r="P7" s="28" t="s">
         <v>156</v>
       </c>
-      <c r="Q7" s="27">
+      <c r="Q7" s="25">
         <v>50</v>
       </c>
-      <c r="R7" s="31">
+      <c r="R7" s="29">
         <v>1</v>
       </c>
-      <c r="S7" s="31">
+      <c r="S7" s="29">
         <v>1</v>
       </c>
-      <c r="T7" s="31">
+      <c r="T7" s="29">
         <v>2</v>
       </c>
-      <c r="U7" s="49">
+      <c r="U7" s="45">
         <v>3</v>
       </c>
-      <c r="V7" s="94"/>
+      <c r="V7" s="91"/>
       <c r="W7" s="14"/>
-      <c r="X7" s="30" t="s">
+      <c r="X7" s="101" t="s">
         <v>157</v>
       </c>
-      <c r="Y7" s="27"/>
-      <c r="Z7" s="32"/>
+      <c r="Y7" s="104"/>
+      <c r="Z7" s="107"/>
       <c r="AA7" s="14"/>
-      <c r="AB7" s="33">
+      <c r="AB7" s="30">
         <v>5</v>
       </c>
-      <c r="AC7" s="35">
+      <c r="AC7" s="32">
         <v>180</v>
       </c>
       <c r="AD7" s="14"/>
-      <c r="AE7" s="52">
+      <c r="AE7" s="48">
         <v>5</v>
       </c>
-      <c r="AF7" s="25" t="s">
+      <c r="AF7" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="AG7" s="53" t="s">
+      <c r="AG7" s="49" t="s">
         <v>165</v>
       </c>
       <c r="AH7" s="14"/>
-      <c r="AI7" s="36" t="s">
+      <c r="AI7" s="33" t="s">
         <v>166</v>
       </c>
       <c r="AJ7" s="14"/>
-      <c r="AK7" s="76">
+      <c r="AK7" s="71">
         <v>5</v>
       </c>
-      <c r="AL7" s="77" t="s">
+      <c r="AL7" s="72" t="s">
         <v>167</v>
       </c>
       <c r="AM7" s="14"/>
-      <c r="AN7" s="76">
+      <c r="AN7" s="71">
         <v>5</v>
       </c>
-      <c r="AO7" s="84" t="s">
+      <c r="AO7" s="79" t="s">
         <v>168</v>
       </c>
       <c r="AP7" s="14"/>
@@ -6029,78 +6134,78 @@
       <c r="G8" s="14"/>
       <c r="H8" s="14"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="28">
+      <c r="J8" s="26">
         <v>5</v>
       </c>
-      <c r="K8" s="29" t="s">
+      <c r="K8" s="27" t="s">
         <v>162</v>
       </c>
       <c r="L8" s="14"/>
-      <c r="M8" s="28">
+      <c r="M8" s="26">
         <v>5</v>
       </c>
-      <c r="N8" s="29" t="s">
+      <c r="N8" s="27" t="s">
         <v>122</v>
       </c>
       <c r="O8" s="14"/>
-      <c r="P8" s="30" t="s">
+      <c r="P8" s="28" t="s">
         <v>163</v>
       </c>
-      <c r="Q8" s="27">
+      <c r="Q8" s="25">
         <v>80</v>
       </c>
-      <c r="R8" s="31">
+      <c r="R8" s="29">
         <v>1</v>
       </c>
-      <c r="S8" s="31">
+      <c r="S8" s="29">
         <v>2</v>
       </c>
-      <c r="T8" s="31">
+      <c r="T8" s="29">
         <v>3</v>
       </c>
-      <c r="U8" s="49">
+      <c r="U8" s="45">
         <v>5</v>
       </c>
-      <c r="V8" s="94"/>
+      <c r="V8" s="91"/>
       <c r="W8" s="14"/>
-      <c r="X8" s="30" t="s">
+      <c r="X8" s="101" t="s">
         <v>164</v>
       </c>
-      <c r="Y8" s="27"/>
-      <c r="Z8" s="32"/>
+      <c r="Y8" s="104"/>
+      <c r="Z8" s="107"/>
       <c r="AA8" s="14"/>
-      <c r="AB8" s="33">
+      <c r="AB8" s="30">
         <v>6</v>
       </c>
-      <c r="AC8" s="35">
+      <c r="AC8" s="32">
         <v>220</v>
       </c>
       <c r="AD8" s="14"/>
-      <c r="AE8" s="52">
+      <c r="AE8" s="48">
         <v>6</v>
       </c>
-      <c r="AF8" s="25" t="s">
+      <c r="AF8" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="AG8" s="53" t="s">
+      <c r="AG8" s="49" t="s">
         <v>173</v>
       </c>
       <c r="AH8" s="14"/>
-      <c r="AI8" s="36" t="s">
+      <c r="AI8" s="33" t="s">
         <v>174</v>
       </c>
       <c r="AJ8" s="14"/>
-      <c r="AK8" s="76">
+      <c r="AK8" s="71">
         <v>6</v>
       </c>
-      <c r="AL8" s="77" t="s">
+      <c r="AL8" s="72" t="s">
         <v>175</v>
       </c>
       <c r="AM8" s="14"/>
-      <c r="AN8" s="76">
+      <c r="AN8" s="71">
         <v>6</v>
       </c>
-      <c r="AO8" s="84" t="s">
+      <c r="AO8" s="79" t="s">
         <v>176</v>
       </c>
       <c r="AP8" s="14"/>
@@ -6109,78 +6214,78 @@
       <c r="G9" s="14"/>
       <c r="H9" s="14"/>
       <c r="I9" s="14"/>
-      <c r="J9" s="28">
+      <c r="J9" s="26">
         <v>6</v>
       </c>
-      <c r="K9" s="29" t="s">
+      <c r="K9" s="27" t="s">
         <v>169</v>
       </c>
       <c r="L9" s="14"/>
-      <c r="M9" s="28">
+      <c r="M9" s="26">
         <v>6</v>
       </c>
-      <c r="N9" s="29" t="s">
+      <c r="N9" s="27" t="s">
         <v>170</v>
       </c>
       <c r="O9" s="14"/>
-      <c r="P9" s="30" t="s">
+      <c r="P9" s="28" t="s">
         <v>171</v>
       </c>
-      <c r="Q9" s="27">
+      <c r="Q9" s="25">
         <v>125</v>
       </c>
-      <c r="R9" s="31">
+      <c r="R9" s="29">
         <v>2</v>
       </c>
-      <c r="S9" s="31">
+      <c r="S9" s="29">
         <v>3</v>
       </c>
-      <c r="T9" s="31">
+      <c r="T9" s="29">
         <v>5</v>
       </c>
-      <c r="U9" s="49">
+      <c r="U9" s="45">
         <v>7</v>
       </c>
-      <c r="V9" s="94"/>
+      <c r="V9" s="91"/>
       <c r="W9" s="14"/>
-      <c r="X9" s="38" t="s">
+      <c r="X9" s="101" t="s">
         <v>172</v>
       </c>
-      <c r="Y9" s="39"/>
-      <c r="Z9" s="40"/>
+      <c r="Y9" s="105"/>
+      <c r="Z9" s="108"/>
       <c r="AA9" s="14"/>
-      <c r="AB9" s="41">
+      <c r="AB9" s="37">
         <v>7</v>
       </c>
-      <c r="AC9" s="43">
+      <c r="AC9" s="39">
         <v>312</v>
       </c>
       <c r="AD9" s="14"/>
-      <c r="AE9" s="52">
+      <c r="AE9" s="48">
         <v>7</v>
       </c>
-      <c r="AF9" s="25" t="s">
+      <c r="AF9" s="23" t="s">
         <v>180</v>
       </c>
-      <c r="AG9" s="53" t="s">
+      <c r="AG9" s="49" t="s">
         <v>139</v>
       </c>
       <c r="AH9" s="14"/>
-      <c r="AI9" s="36" t="s">
+      <c r="AI9" s="33" t="s">
         <v>181</v>
       </c>
       <c r="AJ9" s="14"/>
-      <c r="AK9" s="76">
+      <c r="AK9" s="71">
         <v>7</v>
       </c>
-      <c r="AL9" s="77" t="s">
+      <c r="AL9" s="72" t="s">
         <v>182</v>
       </c>
       <c r="AM9" s="14"/>
-      <c r="AN9" s="78">
+      <c r="AN9" s="73">
         <v>7</v>
       </c>
-      <c r="AO9" s="85" t="s">
+      <c r="AO9" s="80" t="s">
         <v>183</v>
       </c>
       <c r="AP9" s="14"/>
@@ -6189,39 +6294,39 @@
       <c r="G10" s="14"/>
       <c r="H10" s="14"/>
       <c r="I10" s="14"/>
-      <c r="J10" s="28">
+      <c r="J10" s="26">
         <v>7</v>
       </c>
-      <c r="K10" s="29" t="s">
+      <c r="K10" s="27" t="s">
         <v>177</v>
       </c>
       <c r="L10" s="14"/>
-      <c r="M10" s="28">
+      <c r="M10" s="26">
         <v>7</v>
       </c>
-      <c r="N10" s="29" t="s">
+      <c r="N10" s="27" t="s">
         <v>178</v>
       </c>
       <c r="O10" s="14"/>
-      <c r="P10" s="30" t="s">
+      <c r="P10" s="28" t="s">
         <v>179</v>
       </c>
-      <c r="Q10" s="27">
+      <c r="Q10" s="25">
         <v>200</v>
       </c>
-      <c r="R10" s="31">
+      <c r="R10" s="29">
         <v>3</v>
       </c>
-      <c r="S10" s="31">
+      <c r="S10" s="29">
         <v>5</v>
       </c>
-      <c r="T10" s="31">
+      <c r="T10" s="29">
         <v>7</v>
       </c>
-      <c r="U10" s="49">
+      <c r="U10" s="45">
         <v>10</v>
       </c>
-      <c r="V10" s="94"/>
+      <c r="V10" s="91"/>
       <c r="W10" s="14"/>
       <c r="X10" s="14"/>
       <c r="Y10" s="14"/>
@@ -6230,24 +6335,24 @@
       <c r="AB10" s="14"/>
       <c r="AC10" s="14"/>
       <c r="AD10" s="14"/>
-      <c r="AE10" s="52">
+      <c r="AE10" s="48">
         <v>8</v>
       </c>
-      <c r="AF10" s="25" t="s">
+      <c r="AF10" s="23" t="s">
         <v>187</v>
       </c>
-      <c r="AG10" s="53" t="s">
+      <c r="AG10" s="49" t="s">
         <v>188</v>
       </c>
       <c r="AH10" s="14"/>
-      <c r="AI10" s="36" t="s">
+      <c r="AI10" s="33" t="s">
         <v>189</v>
       </c>
       <c r="AJ10" s="14"/>
-      <c r="AK10" s="78">
+      <c r="AK10" s="73">
         <v>8</v>
       </c>
-      <c r="AL10" s="79" t="s">
+      <c r="AL10" s="74" t="s">
         <v>190</v>
       </c>
       <c r="AM10" s="14"/>
@@ -6259,39 +6364,39 @@
       <c r="G11" s="14"/>
       <c r="H11" s="14"/>
       <c r="I11" s="14"/>
-      <c r="J11" s="28">
+      <c r="J11" s="26">
         <v>8</v>
       </c>
-      <c r="K11" s="29" t="s">
+      <c r="K11" s="27" t="s">
         <v>184</v>
       </c>
       <c r="L11" s="14"/>
-      <c r="M11" s="28">
+      <c r="M11" s="26">
         <v>8</v>
       </c>
-      <c r="N11" s="29" t="s">
+      <c r="N11" s="27" t="s">
         <v>185</v>
       </c>
       <c r="O11" s="14"/>
-      <c r="P11" s="30" t="s">
+      <c r="P11" s="28" t="s">
         <v>186</v>
       </c>
-      <c r="Q11" s="27">
+      <c r="Q11" s="25">
         <v>315</v>
       </c>
-      <c r="R11" s="31">
+      <c r="R11" s="29">
         <v>5</v>
       </c>
-      <c r="S11" s="31">
+      <c r="S11" s="29">
         <v>7</v>
       </c>
-      <c r="T11" s="31">
+      <c r="T11" s="29">
         <v>10</v>
       </c>
-      <c r="U11" s="49">
+      <c r="U11" s="45">
         <v>14</v>
       </c>
-      <c r="V11" s="94"/>
+      <c r="V11" s="91"/>
       <c r="W11" s="14"/>
       <c r="X11" s="14"/>
       <c r="Y11" s="14"/>
@@ -6300,17 +6405,17 @@
       <c r="AB11" s="14"/>
       <c r="AC11" s="14"/>
       <c r="AD11" s="14"/>
-      <c r="AE11" s="52">
+      <c r="AE11" s="48">
         <v>9</v>
       </c>
-      <c r="AF11" s="25" t="s">
+      <c r="AF11" s="23" t="s">
         <v>194</v>
       </c>
-      <c r="AG11" s="53" t="s">
+      <c r="AG11" s="49" t="s">
         <v>195</v>
       </c>
       <c r="AH11" s="14"/>
-      <c r="AI11" s="36" t="s">
+      <c r="AI11" s="33" t="s">
         <v>196</v>
       </c>
       <c r="AJ11" s="14"/>
@@ -6325,39 +6430,39 @@
       <c r="G12" s="14"/>
       <c r="H12" s="14"/>
       <c r="I12" s="14"/>
-      <c r="J12" s="28">
+      <c r="J12" s="26">
         <v>9</v>
       </c>
-      <c r="K12" s="29" t="s">
+      <c r="K12" s="27" t="s">
         <v>191</v>
       </c>
       <c r="L12" s="14"/>
-      <c r="M12" s="28">
+      <c r="M12" s="26">
         <v>9</v>
       </c>
-      <c r="N12" s="29" t="s">
+      <c r="N12" s="27" t="s">
         <v>192</v>
       </c>
       <c r="O12" s="14"/>
-      <c r="P12" s="38" t="s">
+      <c r="P12" s="35" t="s">
         <v>193</v>
       </c>
-      <c r="Q12" s="39">
+      <c r="Q12" s="36">
         <v>500</v>
       </c>
-      <c r="R12" s="44">
+      <c r="R12" s="40">
         <v>7</v>
       </c>
-      <c r="S12" s="44">
+      <c r="S12" s="40">
         <v>10</v>
       </c>
-      <c r="T12" s="44">
+      <c r="T12" s="40">
         <v>14</v>
       </c>
-      <c r="U12" s="50">
+      <c r="U12" s="46">
         <v>21</v>
       </c>
-      <c r="V12" s="95"/>
+      <c r="V12" s="92"/>
       <c r="W12" s="14"/>
       <c r="X12" s="14"/>
       <c r="Y12" s="14"/>
@@ -6366,17 +6471,17 @@
       <c r="AB12" s="14"/>
       <c r="AC12" s="14"/>
       <c r="AD12" s="14"/>
-      <c r="AE12" s="52">
+      <c r="AE12" s="48">
         <v>10</v>
       </c>
-      <c r="AF12" s="25" t="s">
+      <c r="AF12" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="AG12" s="53" t="s">
+      <c r="AG12" s="49" t="s">
         <v>199</v>
       </c>
       <c r="AH12" s="14"/>
-      <c r="AI12" s="36" t="s">
+      <c r="AI12" s="33" t="s">
         <v>200</v>
       </c>
       <c r="AJ12" s="14"/>
@@ -6391,17 +6496,17 @@
       <c r="G13" s="14"/>
       <c r="H13" s="14"/>
       <c r="I13" s="14"/>
-      <c r="J13" s="28">
+      <c r="J13" s="26">
         <v>10</v>
       </c>
-      <c r="K13" s="29" t="s">
+      <c r="K13" s="27" t="s">
         <v>197</v>
       </c>
       <c r="L13" s="14"/>
-      <c r="M13" s="28">
+      <c r="M13" s="26">
         <v>10</v>
       </c>
-      <c r="N13" s="29" t="s">
+      <c r="N13" s="27" t="s">
         <v>198</v>
       </c>
       <c r="O13" s="14"/>
@@ -6420,17 +6525,17 @@
       <c r="AB13" s="14"/>
       <c r="AC13" s="14"/>
       <c r="AD13" s="14"/>
-      <c r="AE13" s="52">
+      <c r="AE13" s="48">
         <v>11</v>
       </c>
-      <c r="AF13" s="25" t="s">
+      <c r="AF13" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="AG13" s="53" t="s">
+      <c r="AG13" s="49" t="s">
         <v>203</v>
       </c>
       <c r="AH13" s="14"/>
-      <c r="AI13" s="45" t="s">
+      <c r="AI13" s="41" t="s">
         <v>204</v>
       </c>
       <c r="AJ13" s="14"/>
@@ -6445,17 +6550,17 @@
       <c r="G14" s="14"/>
       <c r="H14" s="14"/>
       <c r="I14" s="14"/>
-      <c r="J14" s="28">
+      <c r="J14" s="26">
         <v>11</v>
       </c>
-      <c r="K14" s="29" t="s">
+      <c r="K14" s="27" t="s">
         <v>201</v>
       </c>
       <c r="L14" s="14"/>
-      <c r="M14" s="28">
+      <c r="M14" s="26">
         <v>11</v>
       </c>
-      <c r="N14" s="29" t="s">
+      <c r="N14" s="27" t="s">
         <v>202</v>
       </c>
       <c r="O14" s="14"/>
@@ -6474,13 +6579,13 @@
       <c r="AB14" s="14"/>
       <c r="AC14" s="14"/>
       <c r="AD14" s="14"/>
-      <c r="AE14" s="52">
+      <c r="AE14" s="48">
         <v>12</v>
       </c>
-      <c r="AF14" s="25" t="s">
+      <c r="AF14" s="23" t="s">
         <v>207</v>
       </c>
-      <c r="AG14" s="53" t="s">
+      <c r="AG14" s="49" t="s">
         <v>208</v>
       </c>
       <c r="AH14" s="14"/>
@@ -6497,15 +6602,15 @@
       <c r="G15" s="14"/>
       <c r="H15" s="14"/>
       <c r="I15" s="14"/>
-      <c r="J15" s="28">
+      <c r="J15" s="26">
         <v>12</v>
       </c>
-      <c r="K15" s="29" t="s">
+      <c r="K15" s="27" t="s">
         <v>205</v>
       </c>
       <c r="L15" s="14"/>
-      <c r="M15" s="28"/>
-      <c r="N15" s="46" t="s">
+      <c r="M15" s="26"/>
+      <c r="N15" s="42" t="s">
         <v>206</v>
       </c>
       <c r="O15" s="14"/>
@@ -6524,13 +6629,13 @@
       <c r="AB15" s="14"/>
       <c r="AC15" s="14"/>
       <c r="AD15" s="14"/>
-      <c r="AE15" s="52">
+      <c r="AE15" s="48">
         <v>13</v>
       </c>
-      <c r="AF15" s="25" t="s">
+      <c r="AF15" s="23" t="s">
         <v>211</v>
       </c>
-      <c r="AG15" s="53" t="s">
+      <c r="AG15" s="49" t="s">
         <v>212</v>
       </c>
       <c r="AH15" s="14"/>
@@ -6547,17 +6652,17 @@
       <c r="G16" s="14"/>
       <c r="H16" s="14"/>
       <c r="I16" s="14"/>
-      <c r="J16" s="37">
+      <c r="J16" s="34">
         <v>13</v>
       </c>
-      <c r="K16" s="47" t="s">
+      <c r="K16" s="43" t="s">
         <v>209</v>
       </c>
       <c r="L16" s="14"/>
-      <c r="M16" s="28">
+      <c r="M16" s="26">
         <v>12</v>
       </c>
-      <c r="N16" s="29" t="s">
+      <c r="N16" s="27" t="s">
         <v>210</v>
       </c>
       <c r="O16" s="13"/>
@@ -6576,13 +6681,13 @@
       <c r="AB16" s="14"/>
       <c r="AC16" s="14"/>
       <c r="AD16" s="14"/>
-      <c r="AE16" s="52">
+      <c r="AE16" s="48">
         <v>14</v>
       </c>
-      <c r="AF16" s="25" t="s">
+      <c r="AF16" s="23" t="s">
         <v>214</v>
       </c>
-      <c r="AG16" s="53" t="s">
+      <c r="AG16" s="49" t="s">
         <v>215</v>
       </c>
       <c r="AH16" s="14"/>
@@ -6602,10 +6707,10 @@
       <c r="J17" s="14"/>
       <c r="K17" s="14"/>
       <c r="L17" s="14"/>
-      <c r="M17" s="28">
+      <c r="M17" s="26">
         <v>13</v>
       </c>
-      <c r="N17" s="29" t="s">
+      <c r="N17" s="27" t="s">
         <v>213</v>
       </c>
       <c r="O17" s="14"/>
@@ -6624,13 +6729,13 @@
       <c r="AB17" s="14"/>
       <c r="AC17" s="14"/>
       <c r="AD17" s="14"/>
-      <c r="AE17" s="52">
+      <c r="AE17" s="48">
         <v>15</v>
       </c>
-      <c r="AF17" s="25" t="s">
+      <c r="AF17" s="23" t="s">
         <v>217</v>
       </c>
-      <c r="AG17" s="53" t="s">
+      <c r="AG17" s="49" t="s">
         <v>218</v>
       </c>
       <c r="AH17" s="14"/>
@@ -6650,10 +6755,10 @@
       <c r="J18" s="14"/>
       <c r="K18" s="14"/>
       <c r="L18" s="14"/>
-      <c r="M18" s="28">
+      <c r="M18" s="26">
         <v>14</v>
       </c>
-      <c r="N18" s="29" t="s">
+      <c r="N18" s="27" t="s">
         <v>216</v>
       </c>
       <c r="O18" s="14"/>
@@ -6672,13 +6777,13 @@
       <c r="AB18" s="14"/>
       <c r="AC18" s="14"/>
       <c r="AD18" s="14"/>
-      <c r="AE18" s="52">
+      <c r="AE18" s="48">
         <v>16</v>
       </c>
-      <c r="AF18" s="25" t="s">
+      <c r="AF18" s="23" t="s">
         <v>220</v>
       </c>
-      <c r="AG18" s="53" t="s">
+      <c r="AG18" s="49" t="s">
         <v>129</v>
       </c>
       <c r="AH18" s="14"/>
@@ -6698,10 +6803,10 @@
       <c r="J19" s="14"/>
       <c r="K19" s="14"/>
       <c r="L19" s="14"/>
-      <c r="M19" s="28">
+      <c r="M19" s="26">
         <v>15</v>
       </c>
-      <c r="N19" s="29" t="s">
+      <c r="N19" s="27" t="s">
         <v>219</v>
       </c>
       <c r="O19" s="14"/>
@@ -6720,13 +6825,13 @@
       <c r="AB19" s="14"/>
       <c r="AC19" s="14"/>
       <c r="AD19" s="14"/>
-      <c r="AE19" s="52">
+      <c r="AE19" s="48">
         <v>17</v>
       </c>
-      <c r="AF19" s="25" t="s">
+      <c r="AF19" s="23" t="s">
         <v>222</v>
       </c>
-      <c r="AG19" s="53" t="s">
+      <c r="AG19" s="49" t="s">
         <v>223</v>
       </c>
       <c r="AH19" s="14"/>
@@ -6746,10 +6851,10 @@
       <c r="J20" s="14"/>
       <c r="K20" s="14"/>
       <c r="L20" s="14"/>
-      <c r="M20" s="28">
+      <c r="M20" s="26">
         <v>16</v>
       </c>
-      <c r="N20" s="29" t="s">
+      <c r="N20" s="27" t="s">
         <v>221</v>
       </c>
       <c r="O20" s="14"/>
@@ -6768,13 +6873,13 @@
       <c r="AB20" s="14"/>
       <c r="AC20" s="14"/>
       <c r="AD20" s="14"/>
-      <c r="AE20" s="52">
+      <c r="AE20" s="48">
         <v>18</v>
       </c>
-      <c r="AF20" s="25" t="s">
+      <c r="AF20" s="23" t="s">
         <v>225</v>
       </c>
-      <c r="AG20" s="53" t="s">
+      <c r="AG20" s="49" t="s">
         <v>226</v>
       </c>
       <c r="AH20" s="14"/>
@@ -6794,10 +6899,10 @@
       <c r="J21" s="14"/>
       <c r="K21" s="14"/>
       <c r="L21" s="14"/>
-      <c r="M21" s="28">
+      <c r="M21" s="26">
         <v>17</v>
       </c>
-      <c r="N21" s="29" t="s">
+      <c r="N21" s="27" t="s">
         <v>224</v>
       </c>
       <c r="O21" s="14"/>
@@ -6816,13 +6921,13 @@
       <c r="AB21" s="14"/>
       <c r="AC21" s="14"/>
       <c r="AD21" s="14"/>
-      <c r="AE21" s="52">
+      <c r="AE21" s="48">
         <v>19</v>
       </c>
-      <c r="AF21" s="25" t="s">
+      <c r="AF21" s="23" t="s">
         <v>228</v>
       </c>
-      <c r="AG21" s="53" t="s">
+      <c r="AG21" s="49" t="s">
         <v>229</v>
       </c>
       <c r="AH21" s="14"/>
@@ -6842,10 +6947,10 @@
       <c r="J22" s="14"/>
       <c r="K22" s="14"/>
       <c r="L22" s="14"/>
-      <c r="M22" s="28">
+      <c r="M22" s="26">
         <v>18</v>
       </c>
-      <c r="N22" s="29" t="s">
+      <c r="N22" s="27" t="s">
         <v>227</v>
       </c>
       <c r="O22" s="14"/>
@@ -6864,13 +6969,13 @@
       <c r="AB22" s="14"/>
       <c r="AC22" s="14"/>
       <c r="AD22" s="14"/>
-      <c r="AE22" s="52">
+      <c r="AE22" s="48">
         <v>20</v>
       </c>
-      <c r="AF22" s="25" t="s">
+      <c r="AF22" s="23" t="s">
         <v>230</v>
       </c>
-      <c r="AG22" s="53" t="s">
+      <c r="AG22" s="49" t="s">
         <v>231</v>
       </c>
       <c r="AH22" s="14"/>
@@ -6890,10 +6995,10 @@
       <c r="J23" s="14"/>
       <c r="K23" s="14"/>
       <c r="L23" s="14"/>
-      <c r="M23" s="28">
+      <c r="M23" s="26">
         <v>19</v>
       </c>
-      <c r="N23" s="47" t="s">
+      <c r="N23" s="43" t="s">
         <v>209</v>
       </c>
       <c r="O23" s="14"/>
@@ -6912,13 +7017,13 @@
       <c r="AB23" s="14"/>
       <c r="AC23" s="14"/>
       <c r="AD23" s="14"/>
-      <c r="AE23" s="52">
+      <c r="AE23" s="48">
         <v>21</v>
       </c>
-      <c r="AF23" s="25" t="s">
+      <c r="AF23" s="23" t="s">
         <v>232</v>
       </c>
-      <c r="AG23" s="53" t="s">
+      <c r="AG23" s="49" t="s">
         <v>233</v>
       </c>
       <c r="AH23" s="14"/>
@@ -6956,13 +7061,13 @@
       <c r="AB24" s="14"/>
       <c r="AC24" s="14"/>
       <c r="AD24" s="14"/>
-      <c r="AE24" s="52">
+      <c r="AE24" s="48">
         <v>22</v>
       </c>
-      <c r="AF24" s="25" t="s">
+      <c r="AF24" s="23" t="s">
         <v>234</v>
       </c>
-      <c r="AG24" s="53" t="s">
+      <c r="AG24" s="49" t="s">
         <v>235</v>
       </c>
       <c r="AH24" s="14"/>
@@ -7000,13 +7105,13 @@
       <c r="AB25" s="14"/>
       <c r="AC25" s="14"/>
       <c r="AD25" s="14"/>
-      <c r="AE25" s="52">
+      <c r="AE25" s="48">
         <v>23</v>
       </c>
-      <c r="AF25" s="25" t="s">
+      <c r="AF25" s="23" t="s">
         <v>236</v>
       </c>
-      <c r="AG25" s="53" t="s">
+      <c r="AG25" s="49" t="s">
         <v>237</v>
       </c>
       <c r="AH25" s="14"/>
@@ -7044,13 +7149,13 @@
       <c r="AB26" s="14"/>
       <c r="AC26" s="14"/>
       <c r="AD26" s="14"/>
-      <c r="AE26" s="52">
+      <c r="AE26" s="48">
         <v>24</v>
       </c>
-      <c r="AF26" s="25" t="s">
+      <c r="AF26" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="AG26" s="53" t="s">
+      <c r="AG26" s="49" t="s">
         <v>239</v>
       </c>
       <c r="AH26" s="14"/>
@@ -7088,13 +7193,13 @@
       <c r="AB27" s="14"/>
       <c r="AC27" s="14"/>
       <c r="AD27" s="14"/>
-      <c r="AE27" s="52">
+      <c r="AE27" s="48">
         <v>25</v>
       </c>
-      <c r="AF27" s="25" t="s">
+      <c r="AF27" s="23" t="s">
         <v>240</v>
       </c>
-      <c r="AG27" s="53" t="s">
+      <c r="AG27" s="49" t="s">
         <v>241</v>
       </c>
       <c r="AH27" s="14"/>
@@ -7132,13 +7237,13 @@
       <c r="AB28" s="14"/>
       <c r="AC28" s="14"/>
       <c r="AD28" s="14"/>
-      <c r="AE28" s="52">
+      <c r="AE28" s="48">
         <v>26</v>
       </c>
-      <c r="AF28" s="25" t="s">
+      <c r="AF28" s="23" t="s">
         <v>242</v>
       </c>
-      <c r="AG28" s="53" t="s">
+      <c r="AG28" s="49" t="s">
         <v>243</v>
       </c>
       <c r="AH28" s="14"/>
@@ -7176,13 +7281,13 @@
       <c r="AB29" s="14"/>
       <c r="AC29" s="14"/>
       <c r="AD29" s="14"/>
-      <c r="AE29" s="54">
+      <c r="AE29" s="50">
         <v>27</v>
       </c>
-      <c r="AF29" s="55" t="s">
+      <c r="AF29" s="51" t="s">
         <v>244</v>
       </c>
-      <c r="AG29" s="56" t="s">
+      <c r="AG29" s="52" t="s">
         <v>245</v>
       </c>
       <c r="AH29" s="14"/>
@@ -7295,7 +7400,7 @@
       <c r="AA32" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="10">
     <mergeCell ref="X2:Z2"/>
     <mergeCell ref="V4:V12"/>
     <mergeCell ref="G2:H2"/>
@@ -7304,6 +7409,8 @@
     <mergeCell ref="P2:P3"/>
     <mergeCell ref="Q2:Q3"/>
     <mergeCell ref="R2:U2"/>
+    <mergeCell ref="Y4:Y9"/>
+    <mergeCell ref="Z4:Z9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>